<commit_message>
Use the live Employeers sheet as the studio crew.
Swap the old Андрій roster for Верлинська, Сиченко as team lead, Колесник and Злотко, with the cards and IBANs from SUPERPLAY_MGX_Calculator.

Co-authored-by: lisenbart <lisenbart@gmail.com>
</commit_message>
<xml_diff>
--- a/data/finance/SUPERPLAY_MGX_Calculator.xlsx
+++ b/data/finance/SUPERPLAY_MGX_Calculator.xlsx
@@ -481,7 +481,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="26">
+  <fills count="30">
     <fill>
       <patternFill/>
     </fill>
@@ -626,6 +626,26 @@
         <fgColor rgb="00BFBFBF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C9DAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -655,7 +675,7 @@
     <xf numFmtId="0" fontId="44" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="44" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="166">
+  <cellXfs count="171">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1114,6 +1134,21 @@
     <xf numFmtId="0" fontId="65" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="65" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="27" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="65" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3163,42 +3198,42 @@
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="44" t="n"/>
-      <c r="B6" s="48" t="inlineStr">
+      <c r="B6" s="166" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C6" s="49" t="inlineStr">
+      <c r="C6" s="167" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D6" s="49" t="n"/>
-      <c r="E6" s="50" t="inlineStr">
+      <c r="D6" s="168" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="F6" s="51" t="inlineStr">
+      <c r="E6" s="169" t="inlineStr">
         <is>
           <t>name of bank</t>
         </is>
       </c>
-      <c r="G6" s="52" t="inlineStr">
+      <c r="F6" s="169" t="inlineStr">
         <is>
           <t>bank card</t>
         </is>
       </c>
-      <c r="H6" s="52" t="inlineStr">
+      <c r="G6" s="170" t="inlineStr">
         <is>
           <t>IBAN</t>
         </is>
       </c>
-      <c r="I6" s="52" t="inlineStr">
+      <c r="H6" s="170" t="inlineStr">
         <is>
           <t>ІПН</t>
         </is>
       </c>
+      <c r="I6" s="52" t="n"/>
       <c r="N6" s="47" t="n"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
@@ -3207,38 +3242,24 @@
       </c>
       <c r="B7" s="53" t="inlineStr">
         <is>
-          <t>Лащенко Сергій Олексійович</t>
-        </is>
-      </c>
-      <c r="C7" s="112" t="inlineStr">
-        <is>
-          <t>+380 93 763 1347</t>
-        </is>
-      </c>
+          <t>Анастасі Верлинська - менеджер</t>
+        </is>
+      </c>
+      <c r="C7" s="112" t="n"/>
       <c r="D7" s="55" t="n"/>
-      <c r="E7" s="42" t="inlineStr">
-        <is>
-          <t>lashenko285@gmail.com</t>
-        </is>
-      </c>
+      <c r="E7" s="42" t="n"/>
       <c r="F7" s="53" t="inlineStr">
         <is>
-          <t>Monobank</t>
+          <t>4874070053093694</t>
         </is>
       </c>
       <c r="G7" s="45" t="inlineStr">
         <is>
-          <t>4441111039612886</t>
-        </is>
-      </c>
-      <c r="H7" s="112" t="inlineStr">
-        <is>
-          <t>UA433220010000026202353175173</t>
-        </is>
-      </c>
-      <c r="I7" s="112" t="n">
-        <v>3276811970</v>
-      </c>
+          <t>UA173220010000026202314266322</t>
+        </is>
+      </c>
+      <c r="H7" s="112" t="n"/>
+      <c r="I7" s="112" t="n"/>
       <c r="M7" s="53" t="n"/>
       <c r="N7" s="56" t="n"/>
     </row>
@@ -3248,7 +3269,7 @@
       </c>
       <c r="B8" s="53" t="inlineStr">
         <is>
-          <t>Анастасія Сиченко</t>
+          <t>Анастасія Сиченко - тімлід</t>
         </is>
       </c>
       <c r="C8" s="112" t="inlineStr">
@@ -3256,27 +3277,23 @@
           <t>+380 99 550 5455</t>
         </is>
       </c>
-      <c r="D8" s="57" t="n"/>
+      <c r="D8" s="57" t="inlineStr">
+        <is>
+          <t>cat44cat22@gmail.com</t>
+        </is>
+      </c>
       <c r="E8" s="42" t="inlineStr">
         <is>
-          <t>cat44cat22@gmail.com</t>
+          <t>Monobank</t>
         </is>
       </c>
       <c r="F8" s="53" t="inlineStr">
         <is>
-          <t>Monobank</t>
-        </is>
-      </c>
-      <c r="G8" s="45" t="inlineStr">
-        <is>
           <t>4441114424460887</t>
         </is>
       </c>
-      <c r="H8" s="112" t="inlineStr">
-        <is>
-          <t>UA173220010000026202314266322</t>
-        </is>
-      </c>
+      <c r="G8" s="45" t="n"/>
+      <c r="H8" s="112" t="n"/>
       <c r="M8" s="53" t="n"/>
       <c r="N8" s="56" t="n"/>
     </row>
@@ -3286,109 +3303,107 @@
       </c>
       <c r="B9" s="53" t="inlineStr">
         <is>
-          <t>Андрій Миглін</t>
+          <t>Лащенко Сергій Олексійович</t>
         </is>
       </c>
       <c r="C9" s="112" t="inlineStr">
         <is>
-          <t>+380 99 608 9025</t>
+          <t>+380 93 763 1347</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>lashenko285@gmail.com</t>
         </is>
       </c>
       <c r="E9" s="42" t="inlineStr">
         <is>
-          <t>andrii.myhlin@gmail.com</t>
+          <t>Monobank</t>
         </is>
       </c>
       <c r="F9" s="53" t="inlineStr">
         <is>
-          <t>Monobank</t>
+          <t>4441111039612886</t>
         </is>
       </c>
       <c r="G9" s="45" t="inlineStr">
         <is>
-          <t>5168752085544776</t>
+          <t>UA433220010000026202353175173</t>
         </is>
       </c>
       <c r="H9" s="112" t="inlineStr">
         <is>
-          <t>UA643052990000026201875784751</t>
-        </is>
-      </c>
-      <c r="I9" s="112" t="n">
-        <v>3734505291</v>
-      </c>
+          <t>3276811970</t>
+        </is>
+      </c>
+      <c r="I9" s="112" t="n"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="140" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B10" s="53" t="inlineStr">
         <is>
           <t>Терлецька Марія Максимівна</t>
         </is>
       </c>
-      <c r="E10" s="43" t="n"/>
-      <c r="F10" s="141" t="inlineStr">
+      <c r="E10" s="43" t="inlineStr">
         <is>
           <t>Monobank</t>
         </is>
       </c>
+      <c r="F10" s="141" t="n"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>UA683220010000026202353816766</t>
+        </is>
+      </c>
       <c r="H10" s="112" t="inlineStr">
         <is>
-          <t>UA683220010000026202353816766</t>
-        </is>
-      </c>
-      <c r="I10" s="112" t="n">
-        <v>3781707605</v>
-      </c>
+          <t>3781707605</t>
+        </is>
+      </c>
+      <c r="I10" s="112" t="n"/>
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="46" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B11" s="53" t="inlineStr">
         <is>
-          <t>Лавренишин Анатлоій</t>
+          <t>Аліна Колесник</t>
         </is>
       </c>
       <c r="C11" s="54" t="n"/>
       <c r="E11" s="43" t="n"/>
-      <c r="F11" s="141" t="inlineStr">
-        <is>
-          <t>Приват</t>
-        </is>
-      </c>
-      <c r="H11" s="112" t="inlineStr">
-        <is>
-          <t>UA433052990000026207663260641</t>
-        </is>
-      </c>
+      <c r="F11" s="141" t="n"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>UA193220010000026205327095598</t>
+        </is>
+      </c>
+      <c r="H11" s="112" t="n"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" t="n">
+        <v>7</v>
+      </c>
       <c r="B12" s="150" t="inlineStr">
         <is>
-          <t>Маргарита Бездітко</t>
-        </is>
-      </c>
-      <c r="C12" s="151" t="inlineStr">
-        <is>
-          <t>+380 73 123 0042</t>
-        </is>
-      </c>
+          <t>Злотко Олексій</t>
+        </is>
+      </c>
+      <c r="C12" s="151" t="n"/>
       <c r="D12" s="152" t="n"/>
-      <c r="E12" s="152" t="inlineStr">
-        <is>
-          <t>rita.bezditko@gmail.com</t>
-        </is>
-      </c>
+      <c r="E12" s="152" t="n"/>
       <c r="F12" s="150" t="inlineStr">
         <is>
-          <t>Monobank</t>
+          <t>432345037851582</t>
         </is>
       </c>
       <c r="G12" s="153" t="inlineStr">
         <is>
-          <t>4441114427187438</t>
+          <t>UA943077700000026208713943056</t>
         </is>
       </c>
     </row>
@@ -3405,7 +3420,7 @@
       <c r="B16" s="56" t="n"/>
       <c r="D16" s="43" t="n"/>
       <c r="E16" s="43" t="n"/>
-      <c r="H16" s="137" t="inlineStr"/>
+      <c r="H16" s="137" t="n"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="B17" s="56" t="n"/>

</xml_diff>

<commit_message>
Make Studio tax editable and persist it in the calculator.
TAX % sits on the STUDIO (TAX) row, defaults to 6%, and rewriting the calculator stores the rate in a TAX cell the formulas use.

Co-authored-by: lisenbart <lisenbart@gmail.com>
</commit_message>
<xml_diff>
--- a/data/finance/SUPERPLAY_MGX_Calculator.xlsx
+++ b/data/finance/SUPERPLAY_MGX_Calculator.xlsx
@@ -481,7 +481,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="30">
+  <fills count="33">
     <fill>
       <patternFill/>
     </fill>
@@ -646,6 +646,21 @@
         <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="009d50dd"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6B19B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B4A7D6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -675,7 +690,7 @@
     <xf numFmtId="0" fontId="44" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="44" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="171">
+  <cellXfs count="175">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1149,6 +1164,18 @@
     <xf numFmtId="49" fontId="65" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="66" fillId="30" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="66" fillId="31" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="66" fillId="32" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="65" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1362,7 +1389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:P34"/>
+  <dimension ref="A2:Q36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1381,6 +1408,7 @@
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1391,32 +1419,32 @@
       </c>
       <c r="F2" s="156" t="inlineStr">
         <is>
+          <t>Анастасія</t>
+        </is>
+      </c>
+      <c r="G2" s="156" t="inlineStr">
+        <is>
           <t>Настя</t>
         </is>
       </c>
-      <c r="G2" s="156" t="inlineStr">
+      <c r="H2" s="156" t="inlineStr">
+        <is>
+          <t>Сергій</t>
+        </is>
+      </c>
+      <c r="I2" s="156" t="inlineStr">
         <is>
           <t>Маша</t>
         </is>
       </c>
-      <c r="H2" s="156" t="inlineStr">
-        <is>
-          <t>Сергій</t>
-        </is>
-      </c>
-      <c r="I2" s="156" t="inlineStr">
+      <c r="J2" s="156" t="inlineStr">
         <is>
           <t>Аліна</t>
         </is>
       </c>
-      <c r="J2" s="156" t="inlineStr">
+      <c r="K2" s="156" t="inlineStr">
         <is>
           <t>Олекса</t>
-        </is>
-      </c>
-      <c r="K2" s="156" t="inlineStr">
-        <is>
-          <t>Андрій</t>
         </is>
       </c>
     </row>
@@ -1502,13 +1530,16 @@
         <v/>
       </c>
       <c r="E6" s="159" t="n"/>
-      <c r="F6" s="161">
-        <f>D6*15</f>
+      <c r="F6" s="171">
+        <f>D6*5</f>
         <v/>
       </c>
       <c r="G6" s="159" t="n"/>
       <c r="H6" s="159" t="n"/>
-      <c r="I6" s="159" t="n"/>
+      <c r="I6" s="163">
+        <f>D6*15</f>
+        <v/>
+      </c>
       <c r="J6" s="159" t="n"/>
       <c r="K6" s="159" t="n"/>
       <c r="L6" s="159">
@@ -1535,8 +1566,14 @@
         <v/>
       </c>
       <c r="E7" s="159" t="n"/>
-      <c r="F7" s="159" t="n"/>
-      <c r="G7" s="159" t="n"/>
+      <c r="F7" s="171">
+        <f>D7*5</f>
+        <v/>
+      </c>
+      <c r="G7" s="161">
+        <f>D7*15</f>
+        <v/>
+      </c>
       <c r="H7" s="159" t="n"/>
       <c r="I7" s="159" t="n"/>
       <c r="J7" s="159" t="n"/>
@@ -1565,7 +1602,10 @@
         <v/>
       </c>
       <c r="E8" s="159" t="n"/>
-      <c r="F8" s="159" t="n"/>
+      <c r="F8" s="171">
+        <f>D8*5</f>
+        <v/>
+      </c>
       <c r="G8" s="159" t="n"/>
       <c r="H8" s="162">
         <f>D8*15</f>
@@ -1587,7 +1627,7 @@
       <c r="A9" s="159" t="n"/>
       <c r="B9" s="160" t="inlineStr">
         <is>
-          <t>DX-AIV-0218-002_SettAI_PuzzleHalloween_DX-VEO-055-001_EN_30s</t>
+          <t>DX-AIV-0215-002_SettAI_HallweenSkull_DX-VEO-055-001_EN_30s</t>
         </is>
       </c>
       <c r="C9" s="159" t="n">
@@ -1598,11 +1638,14 @@
         <v/>
       </c>
       <c r="E9" s="159" t="n"/>
-      <c r="F9" s="161">
+      <c r="F9" s="171">
+        <f>D9*5</f>
+        <v/>
+      </c>
+      <c r="G9" s="161">
         <f>D9*15</f>
         <v/>
       </c>
-      <c r="G9" s="159" t="n"/>
       <c r="H9" s="159" t="n"/>
       <c r="I9" s="159" t="n"/>
       <c r="J9" s="159" t="n"/>
@@ -1620,7 +1663,7 @@
       <c r="A10" s="159" t="n"/>
       <c r="B10" s="160" t="inlineStr">
         <is>
-          <t>DX-AIV-0222-003_SettAI_HalloweenRelax_DX-VEO-055-001_EN_30s</t>
+          <t>DX-AIV-0218-002_SettAI_PuzzleHalloween_DX-VEO-055-001_EN_30s</t>
         </is>
       </c>
       <c r="C10" s="159" t="n">
@@ -1631,8 +1674,14 @@
         <v/>
       </c>
       <c r="E10" s="159" t="n"/>
-      <c r="F10" s="159" t="n"/>
-      <c r="G10" s="159" t="n"/>
+      <c r="F10" s="171">
+        <f>D10*5</f>
+        <v/>
+      </c>
+      <c r="G10" s="161">
+        <f>D10*15</f>
+        <v/>
+      </c>
       <c r="H10" s="159" t="n"/>
       <c r="I10" s="159" t="n"/>
       <c r="J10" s="159" t="n"/>
@@ -1650,7 +1699,7 @@
       <c r="A11" s="159" t="n"/>
       <c r="B11" s="160" t="inlineStr">
         <is>
-          <t>DX-AIV-0225-002_SettAI_HalloweenSave_DX-VEO-055-001_EN_60s</t>
+          <t>DX-AIV-0222-003_SettAI_HalloweenRelax_DX-VEO-055-001_EN_30s</t>
         </is>
       </c>
       <c r="C11" s="159" t="n">
@@ -1661,11 +1710,14 @@
         <v/>
       </c>
       <c r="E11" s="159" t="n"/>
-      <c r="F11" s="161">
+      <c r="F11" s="171">
+        <f>D11*5</f>
+        <v/>
+      </c>
+      <c r="G11" s="161">
         <f>D11*15</f>
         <v/>
       </c>
-      <c r="G11" s="159" t="n"/>
       <c r="H11" s="159" t="n"/>
       <c r="I11" s="159" t="n"/>
       <c r="J11" s="159" t="n"/>
@@ -1683,7 +1735,7 @@
       <c r="A12" s="159" t="n"/>
       <c r="B12" s="160" t="inlineStr">
         <is>
-          <t>DX-AIV-0230-002_SettAI_HalloweenTower_ DX-VEO-055-001 _EN_60s</t>
+          <t>DX-AIV-0225-002_SettAI_HalloweenSave_DX-VEO-055-001_EN_60</t>
         </is>
       </c>
       <c r="C12" s="159" t="n">
@@ -1694,13 +1746,16 @@
         <v/>
       </c>
       <c r="E12" s="159" t="n"/>
-      <c r="F12" s="159" t="n"/>
-      <c r="G12" s="163">
-        <f>D12*12</f>
-        <v/>
-      </c>
+      <c r="F12" s="171">
+        <f>D12*5</f>
+        <v/>
+      </c>
+      <c r="G12" s="159" t="n"/>
       <c r="H12" s="159" t="n"/>
-      <c r="I12" s="159" t="n"/>
+      <c r="I12" s="163">
+        <f>D12*15</f>
+        <v/>
+      </c>
       <c r="J12" s="159" t="n"/>
       <c r="K12" s="159" t="n"/>
       <c r="L12" s="159">
@@ -1716,7 +1771,7 @@
       <c r="A13" s="159" t="n"/>
       <c r="B13" s="160" t="inlineStr">
         <is>
-          <t>DX-AIV-0406-002_SettAI_InteractiveHalloween_DX-VEO-055-001_EN_60s</t>
+          <t>DX-AIV-0225-002_SettAI_HalloweenSave_DX-VEO-055-001_EN_60s</t>
         </is>
       </c>
       <c r="C13" s="159" t="n">
@@ -1727,9 +1782,12 @@
         <v/>
       </c>
       <c r="E13" s="159" t="n"/>
-      <c r="F13" s="159" t="n"/>
-      <c r="G13" s="163">
-        <f>D13*12</f>
+      <c r="F13" s="171">
+        <f>D13*5</f>
+        <v/>
+      </c>
+      <c r="G13" s="161">
+        <f>D13*15</f>
         <v/>
       </c>
       <c r="H13" s="159" t="n"/>
@@ -1749,7 +1807,7 @@
       <c r="A14" s="159" t="n"/>
       <c r="B14" s="160" t="inlineStr">
         <is>
-          <t>DX-AIV-0407-002_SettAI_GraveEscape_DX-VEO-055-001_EN_60s</t>
+          <t>DX-AIV-0230-002_SettAI_HalloweenTower_ DX-VEO-055-001 _EN_60s</t>
         </is>
       </c>
       <c r="C14" s="159" t="n">
@@ -1760,13 +1818,16 @@
         <v/>
       </c>
       <c r="E14" s="159" t="n"/>
-      <c r="F14" s="159" t="n"/>
-      <c r="G14" s="163">
-        <f>D14*12</f>
-        <v/>
-      </c>
+      <c r="F14" s="171">
+        <f>D14*5</f>
+        <v/>
+      </c>
+      <c r="G14" s="159" t="n"/>
       <c r="H14" s="159" t="n"/>
-      <c r="I14" s="159" t="n"/>
+      <c r="I14" s="163">
+        <f>D14*15</f>
+        <v/>
+      </c>
       <c r="J14" s="159" t="n"/>
       <c r="K14" s="159" t="n"/>
       <c r="L14" s="159">
@@ -1782,7 +1843,7 @@
       <c r="A15" s="159" t="n"/>
       <c r="B15" s="160" t="inlineStr">
         <is>
-          <t>DX-AIV-216-002_SettAI_HalloweenCircle_DX-VEO-055-001_EN_60s</t>
+          <t>DX-AIV-0406-002_SettAI_InteractiveHalloween_DX-VEO-055-001_EN_60s</t>
         </is>
       </c>
       <c r="C15" s="159" t="n">
@@ -1793,13 +1854,16 @@
         <v/>
       </c>
       <c r="E15" s="159" t="n"/>
-      <c r="F15" s="161">
-        <f>D15*15</f>
+      <c r="F15" s="171">
+        <f>D15*5</f>
         <v/>
       </c>
       <c r="G15" s="159" t="n"/>
       <c r="H15" s="159" t="n"/>
-      <c r="I15" s="159" t="n"/>
+      <c r="I15" s="163">
+        <f>D15*15</f>
+        <v/>
+      </c>
       <c r="J15" s="159" t="n"/>
       <c r="K15" s="159" t="n"/>
       <c r="L15" s="159">
@@ -1815,7 +1879,7 @@
       <c r="A16" s="159" t="n"/>
       <c r="B16" s="160" t="inlineStr">
         <is>
-          <t>DX-AIV-231-002_SettAI_Halloween_Spirals_DX-VEO-055-001_EN_60s</t>
+          <t>DX-AIV-0407-002_SettAI_GraveEscape_DX-VEO-055-001_EN_60s</t>
         </is>
       </c>
       <c r="C16" s="159" t="n">
@@ -1826,10 +1890,16 @@
         <v/>
       </c>
       <c r="E16" s="159" t="n"/>
-      <c r="F16" s="159" t="n"/>
+      <c r="F16" s="171">
+        <f>D16*5</f>
+        <v/>
+      </c>
       <c r="G16" s="159" t="n"/>
       <c r="H16" s="159" t="n"/>
-      <c r="I16" s="159" t="n"/>
+      <c r="I16" s="163">
+        <f>D16*15</f>
+        <v/>
+      </c>
       <c r="J16" s="159" t="n"/>
       <c r="K16" s="159" t="n"/>
       <c r="L16" s="159">
@@ -1841,141 +1911,150 @@
         <v/>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="159" t="n"/>
+      <c r="B17" s="160" t="inlineStr">
+        <is>
+          <t>DX-AIV-216-002_SettAI_HalloweenCircle_DX-VEO-055-001_EN_60s</t>
+        </is>
+      </c>
+      <c r="C17" s="159" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D17" s="159">
+        <f>C17*9</f>
+        <v/>
+      </c>
+      <c r="E17" s="159" t="n"/>
+      <c r="F17" s="171">
+        <f>D17*5</f>
+        <v/>
+      </c>
+      <c r="G17" s="161">
+        <f>D17*15</f>
+        <v/>
+      </c>
+      <c r="H17" s="159" t="n"/>
+      <c r="I17" s="159" t="n"/>
+      <c r="J17" s="159" t="n"/>
+      <c r="K17" s="159" t="n"/>
+      <c r="L17" s="159">
+        <f>SUM(F17:K17)</f>
+        <v/>
+      </c>
+      <c r="M17" s="159">
+        <f>D17*35</f>
+        <v/>
+      </c>
+    </row>
     <row r="18">
-      <c r="A18" s="164" t="inlineStr">
+      <c r="A18" s="159" t="n"/>
+      <c r="B18" s="160" t="inlineStr">
+        <is>
+          <t>DX-AIV-231-002_SettAI_Halloween_Spirals_DX-VEO-055-001_EN_60s</t>
+        </is>
+      </c>
+      <c r="C18" s="159" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D18" s="159">
+        <f>C18*9</f>
+        <v/>
+      </c>
+      <c r="E18" s="159" t="n"/>
+      <c r="F18" s="171">
+        <f>D18*5</f>
+        <v/>
+      </c>
+      <c r="G18" s="159" t="n"/>
+      <c r="H18" s="159" t="n"/>
+      <c r="I18" s="163">
+        <f>D18*15</f>
+        <v/>
+      </c>
+      <c r="J18" s="159" t="n"/>
+      <c r="K18" s="159" t="n"/>
+      <c r="L18" s="159">
+        <f>SUM(F18:K18)</f>
+        <v/>
+      </c>
+      <c r="M18" s="159">
+        <f>D18*35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="164" t="inlineStr">
         <is>
           <t>DD</t>
         </is>
       </c>
-      <c r="B18" s="158" t="inlineStr">
+      <c r="B20" s="158" t="inlineStr">
         <is>
           <t>MGX</t>
         </is>
       </c>
-      <c r="C18" s="158" t="inlineStr">
+      <c r="C20" s="158" t="inlineStr">
         <is>
           <t>SHIFTS</t>
         </is>
       </c>
-      <c r="D18" s="158" t="inlineStr">
+      <c r="D20" s="158" t="inlineStr">
         <is>
           <t>HOURS</t>
         </is>
       </c>
-      <c r="E18" s="158" t="inlineStr">
+      <c r="E20" s="158" t="inlineStr">
         <is>
           <t>D.LINE</t>
         </is>
       </c>
-      <c r="F18" s="158" t="inlineStr">
+      <c r="F20" s="158" t="inlineStr">
         <is>
           <t>EMPL 1</t>
         </is>
       </c>
-      <c r="G18" s="158" t="inlineStr">
+      <c r="G20" s="158" t="inlineStr">
         <is>
           <t>EMPL 2</t>
         </is>
       </c>
-      <c r="H18" s="158" t="inlineStr">
+      <c r="H20" s="158" t="inlineStr">
         <is>
           <t>EMPL 3</t>
         </is>
       </c>
-      <c r="I18" s="158" t="inlineStr">
+      <c r="I20" s="158" t="inlineStr">
         <is>
           <t>EMPL 4</t>
         </is>
       </c>
-      <c r="J18" s="158" t="inlineStr">
+      <c r="J20" s="158" t="inlineStr">
         <is>
           <t>EMPL 5</t>
         </is>
       </c>
-      <c r="K18" s="158" t="inlineStr">
+      <c r="K20" s="158" t="inlineStr">
         <is>
           <t>EMPL 6</t>
         </is>
       </c>
-      <c r="L18" s="158" t="inlineStr">
+      <c r="L20" s="158" t="inlineStr">
         <is>
           <t>Total EMPL</t>
         </is>
       </c>
-      <c r="M18" s="158" t="inlineStr">
+      <c r="M20" s="158" t="inlineStr">
         <is>
           <t>CLIENT IN</t>
         </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="159" t="n"/>
-      <c r="B19" s="160" t="inlineStr">
-        <is>
-          <t>DD-AIV-202-004_SettAI_HalloweenFireTrial_DD-VEO-059-001_EN_30s</t>
-        </is>
-      </c>
-      <c r="C19" s="159" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="D19" s="159">
-        <f>C19*9</f>
-        <v/>
-      </c>
-      <c r="E19" s="159" t="n"/>
-      <c r="F19" s="159" t="n"/>
-      <c r="G19" s="159" t="n"/>
-      <c r="H19" s="159" t="n"/>
-      <c r="I19" s="159" t="n"/>
-      <c r="J19" s="159" t="n"/>
-      <c r="K19" s="159" t="n"/>
-      <c r="L19" s="159">
-        <f>SUM(F19:K19)</f>
-        <v/>
-      </c>
-      <c r="M19" s="159">
-        <f>D19*35</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="159" t="n"/>
-      <c r="B20" s="160" t="inlineStr">
-        <is>
-          <t>DD-AIV-224-002_SettAI_HalloweenMario_DD-VEO-059-001_EN_30s</t>
-        </is>
-      </c>
-      <c r="C20" s="159" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="D20" s="159">
-        <f>C20*9</f>
-        <v/>
-      </c>
-      <c r="E20" s="159" t="n"/>
-      <c r="F20" s="159" t="n"/>
-      <c r="G20" s="163">
-        <f>D20*12</f>
-        <v/>
-      </c>
-      <c r="H20" s="159" t="n"/>
-      <c r="I20" s="159" t="n"/>
-      <c r="J20" s="159" t="n"/>
-      <c r="K20" s="159" t="n"/>
-      <c r="L20" s="159">
-        <f>SUM(F20:K20)</f>
-        <v/>
-      </c>
-      <c r="M20" s="159">
-        <f>D20*35</f>
-        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="159" t="n"/>
       <c r="B21" s="160" t="inlineStr">
         <is>
-          <t>DD-AIV-225-002_SettAI_HalloweenTrap_DD-VEO-059-001_EN_30s</t>
+          <t>DD-AIV-202-004_SettAI_HalloweenFireTrial_DD-VEO-059-001_EN_30s</t>
         </is>
       </c>
       <c r="C21" s="159" t="n">
@@ -1986,13 +2065,16 @@
         <v/>
       </c>
       <c r="E21" s="159" t="n"/>
-      <c r="F21" s="159" t="n"/>
-      <c r="G21" s="163">
-        <f>D21*12</f>
-        <v/>
-      </c>
+      <c r="F21" s="171">
+        <f>D21*5</f>
+        <v/>
+      </c>
+      <c r="G21" s="159" t="n"/>
       <c r="H21" s="159" t="n"/>
-      <c r="I21" s="159" t="n"/>
+      <c r="I21" s="163">
+        <f>D21*15</f>
+        <v/>
+      </c>
       <c r="J21" s="159" t="n"/>
       <c r="K21" s="159" t="n"/>
       <c r="L21" s="159">
@@ -2008,7 +2090,7 @@
       <c r="A22" s="159" t="n"/>
       <c r="B22" s="160" t="inlineStr">
         <is>
-          <t>DD-AIV-227-002_SettAI_HalloweenBlastTreasure_DD-VEO-059-001_EN_24s</t>
+          <t>DD-AIV-224-002_SettAI_HalloweenMario_DD-VEO-059-001_EN_30s</t>
         </is>
       </c>
       <c r="C22" s="159" t="n">
@@ -2019,11 +2101,17 @@
         <v/>
       </c>
       <c r="E22" s="159" t="n"/>
-      <c r="F22" s="159" t="n"/>
+      <c r="F22" s="171">
+        <f>D22*5</f>
+        <v/>
+      </c>
       <c r="G22" s="159" t="n"/>
       <c r="H22" s="159" t="n"/>
       <c r="I22" s="159" t="n"/>
-      <c r="J22" s="159" t="n"/>
+      <c r="J22" s="172">
+        <f>D22*15</f>
+        <v/>
+      </c>
       <c r="K22" s="159" t="n"/>
       <c r="L22" s="159">
         <f>SUM(F22:K22)</f>
@@ -2038,7 +2126,7 @@
       <c r="A23" s="159" t="n"/>
       <c r="B23" s="160" t="inlineStr">
         <is>
-          <t>DD-AIV-228-002_SettAI_HalloweenBlastTreasure_DD-VEO-059-001_EN_30s</t>
+          <t>DD-AIV-225-002_SettAI_HalloweenTrap_DD-VEO-059-001_EN_30s</t>
         </is>
       </c>
       <c r="C23" s="159" t="n">
@@ -2049,11 +2137,17 @@
         <v/>
       </c>
       <c r="E23" s="159" t="n"/>
-      <c r="F23" s="159" t="n"/>
+      <c r="F23" s="171">
+        <f>D23*5</f>
+        <v/>
+      </c>
       <c r="G23" s="159" t="n"/>
       <c r="H23" s="159" t="n"/>
       <c r="I23" s="159" t="n"/>
-      <c r="J23" s="159" t="n"/>
+      <c r="J23" s="172">
+        <f>D23*15</f>
+        <v/>
+      </c>
       <c r="K23" s="159" t="n"/>
       <c r="L23" s="159">
         <f>SUM(F23:K23)</f>
@@ -2068,7 +2162,7 @@
       <c r="A24" s="159" t="n"/>
       <c r="B24" s="160" t="inlineStr">
         <is>
-          <t>DD-AIV-229-002_SettAI_HalloweenMonopoly_DD-VEO-059-001_EN_30s</t>
+          <t>DD-AIV-227-002_SettAI_HalloweenBlastTreasure_DD-VEO-059-001_EN_24s</t>
         </is>
       </c>
       <c r="C24" s="159" t="n">
@@ -2079,10 +2173,16 @@
         <v/>
       </c>
       <c r="E24" s="159" t="n"/>
-      <c r="F24" s="159" t="n"/>
+      <c r="F24" s="171">
+        <f>D24*5</f>
+        <v/>
+      </c>
       <c r="G24" s="159" t="n"/>
       <c r="H24" s="159" t="n"/>
-      <c r="I24" s="159" t="n"/>
+      <c r="I24" s="163">
+        <f>D24*15</f>
+        <v/>
+      </c>
       <c r="J24" s="159" t="n"/>
       <c r="K24" s="159" t="n"/>
       <c r="L24" s="159">
@@ -2098,7 +2198,7 @@
       <c r="A25" s="159" t="n"/>
       <c r="B25" s="160" t="inlineStr">
         <is>
-          <t>DD-AIV-231-002_SettAI_SpookyJackpot_DD-VEO-059-001_EN_30s</t>
+          <t>DD-AIV-228-002_SettAI_HalloweenBlastTreasure_DD-VEO-059-001_EN_30s</t>
         </is>
       </c>
       <c r="C25" s="159" t="n">
@@ -2109,15 +2209,18 @@
         <v/>
       </c>
       <c r="E25" s="159" t="n"/>
-      <c r="F25" s="159" t="n"/>
+      <c r="F25" s="171">
+        <f>D25*5</f>
+        <v/>
+      </c>
       <c r="G25" s="159" t="n"/>
-      <c r="H25" s="162">
-        <f>D25*15</f>
-        <v/>
-      </c>
+      <c r="H25" s="159" t="n"/>
       <c r="I25" s="159" t="n"/>
       <c r="J25" s="159" t="n"/>
-      <c r="K25" s="159" t="n"/>
+      <c r="K25" s="173">
+        <f>D25*15</f>
+        <v/>
+      </c>
       <c r="L25" s="159">
         <f>SUM(F25:K25)</f>
         <v/>
@@ -2131,7 +2234,7 @@
       <c r="A26" s="159" t="n"/>
       <c r="B26" s="160" t="inlineStr">
         <is>
-          <t>DD-AIV-233-002_SettAI_HalloweenKindomBuild_DD-VEO-059-001_EN_60s</t>
+          <t>DD-AIV-229-002_SettAI_HalloweenMonopoly_DD-VEO-059-001_EN_30s</t>
         </is>
       </c>
       <c r="C26" s="159" t="n">
@@ -2142,12 +2245,18 @@
         <v/>
       </c>
       <c r="E26" s="159" t="n"/>
-      <c r="F26" s="159" t="n"/>
+      <c r="F26" s="171">
+        <f>D26*5</f>
+        <v/>
+      </c>
       <c r="G26" s="159" t="n"/>
       <c r="H26" s="159" t="n"/>
       <c r="I26" s="159" t="n"/>
       <c r="J26" s="159" t="n"/>
-      <c r="K26" s="159" t="n"/>
+      <c r="K26" s="173">
+        <f>D26*15</f>
+        <v/>
+      </c>
       <c r="L26" s="159">
         <f>SUM(F26:K26)</f>
         <v/>
@@ -2161,7 +2270,7 @@
       <c r="A27" s="159" t="n"/>
       <c r="B27" s="160" t="inlineStr">
         <is>
-          <t>DD-AIV-235-002_SettAI_WitchsPotion_DD-VEO-059-001_EN_30s</t>
+          <t>DD-AIV-231-002_SettAI_SpookyJackpot_DD-VEO-059-001_EN_30s</t>
         </is>
       </c>
       <c r="C27" s="159" t="n">
@@ -2172,8 +2281,14 @@
         <v/>
       </c>
       <c r="E27" s="159" t="n"/>
-      <c r="F27" s="159" t="n"/>
-      <c r="G27" s="159" t="n"/>
+      <c r="F27" s="171">
+        <f>D27*5</f>
+        <v/>
+      </c>
+      <c r="G27" s="161">
+        <f>D27*15</f>
+        <v/>
+      </c>
       <c r="H27" s="159" t="n"/>
       <c r="I27" s="159" t="n"/>
       <c r="J27" s="159" t="n"/>
@@ -2191,7 +2306,7 @@
       <c r="A28" s="159" t="n"/>
       <c r="B28" s="160" t="inlineStr">
         <is>
-          <t>DD-AIV-239-002_SettAI_HalloweenDiamondBlast_DD-VEO-059-001_EN_30s</t>
+          <t>DD-AIV-233-002_SettAI_HalloweenKindomBuild_DD-VEO-059-001_EN_60s</t>
         </is>
       </c>
       <c r="C28" s="159" t="n">
@@ -2202,10 +2317,16 @@
         <v/>
       </c>
       <c r="E28" s="159" t="n"/>
-      <c r="F28" s="159" t="n"/>
+      <c r="F28" s="171">
+        <f>D28*5</f>
+        <v/>
+      </c>
       <c r="G28" s="159" t="n"/>
       <c r="H28" s="159" t="n"/>
-      <c r="I28" s="159" t="n"/>
+      <c r="I28" s="163">
+        <f>D28*15</f>
+        <v/>
+      </c>
       <c r="J28" s="159" t="n"/>
       <c r="K28" s="159" t="n"/>
       <c r="L28" s="159">
@@ -2217,154 +2338,231 @@
         <v/>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="159" t="n"/>
+      <c r="B29" s="160" t="inlineStr">
+        <is>
+          <t>DD-AIV-235-002_SettAI_WitchsPotion_DD-VEO-059-001_EN_30s</t>
+        </is>
+      </c>
+      <c r="C29" s="159" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D29" s="159">
+        <f>C29*9</f>
+        <v/>
+      </c>
+      <c r="E29" s="159" t="n"/>
+      <c r="F29" s="171">
+        <f>D29*5</f>
+        <v/>
+      </c>
+      <c r="G29" s="159" t="n"/>
+      <c r="H29" s="159" t="n"/>
+      <c r="I29" s="159" t="n"/>
+      <c r="J29" s="159" t="n"/>
+      <c r="K29" s="159" t="n"/>
+      <c r="L29" s="159">
+        <f>SUM(F29:K29)</f>
+        <v/>
+      </c>
+      <c r="M29" s="159">
+        <f>D29*35</f>
+        <v/>
+      </c>
+    </row>
     <row r="30">
-      <c r="A30" s="158" t="inlineStr">
+      <c r="A30" s="159" t="n"/>
+      <c r="B30" s="160" t="inlineStr">
+        <is>
+          <t>DD-AIV-239-002_SettAI_HalloweenDiamondBlast_DD-VEO-059-001_EN_30s</t>
+        </is>
+      </c>
+      <c r="C30" s="159" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D30" s="159">
+        <f>C30*9</f>
+        <v/>
+      </c>
+      <c r="E30" s="159" t="n"/>
+      <c r="F30" s="171">
+        <f>D30*5</f>
+        <v/>
+      </c>
+      <c r="G30" s="161">
+        <f>D30*15</f>
+        <v/>
+      </c>
+      <c r="H30" s="159" t="n"/>
+      <c r="I30" s="159" t="n"/>
+      <c r="J30" s="159" t="n"/>
+      <c r="K30" s="159" t="n"/>
+      <c r="L30" s="159">
+        <f>SUM(F30:K30)</f>
+        <v/>
+      </c>
+      <c r="M30" s="159">
+        <f>D30*35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="158" t="inlineStr">
         <is>
           <t>total</t>
         </is>
       </c>
-      <c r="B30" s="165" t="n"/>
-      <c r="C30" s="158">
-        <f>SUM(C6:C28)</f>
-        <v/>
-      </c>
-      <c r="D30" s="158">
-        <f>SUM(D6:D28)</f>
-        <v/>
-      </c>
-      <c r="E30" s="158" t="n"/>
-      <c r="F30" s="158">
-        <f>SUM(F6:F28)</f>
-        <v/>
-      </c>
-      <c r="G30" s="158">
-        <f>SUM(G6:G28)</f>
-        <v/>
-      </c>
-      <c r="H30" s="158">
-        <f>SUM(H6:H28)</f>
-        <v/>
-      </c>
-      <c r="I30" s="158">
-        <f>SUM(I6:I28)</f>
-        <v/>
-      </c>
-      <c r="J30" s="158">
-        <f>SUM(J6:J28)</f>
-        <v/>
-      </c>
-      <c r="K30" s="158">
-        <f>SUM(K6:K28)</f>
-        <v/>
-      </c>
-      <c r="L30" s="158">
-        <f>SUM(F30:K30)</f>
-        <v/>
-      </c>
-      <c r="M30" s="158">
-        <f>SUM(M6:M28)</f>
-        <v/>
-      </c>
-      <c r="O30" s="155" t="inlineStr">
+      <c r="B32" s="165" t="n"/>
+      <c r="C32" s="158">
+        <f>SUM(C6:C30)</f>
+        <v/>
+      </c>
+      <c r="D32" s="158">
+        <f>SUM(D6:D30)</f>
+        <v/>
+      </c>
+      <c r="E32" s="158" t="n"/>
+      <c r="F32" s="158">
+        <f>SUM(F6:F30)</f>
+        <v/>
+      </c>
+      <c r="G32" s="158">
+        <f>SUM(G6:G30)</f>
+        <v/>
+      </c>
+      <c r="H32" s="158">
+        <f>SUM(H6:H30)</f>
+        <v/>
+      </c>
+      <c r="I32" s="158">
+        <f>SUM(I6:I30)</f>
+        <v/>
+      </c>
+      <c r="J32" s="158">
+        <f>SUM(J6:J30)</f>
+        <v/>
+      </c>
+      <c r="K32" s="158">
+        <f>SUM(K6:K30)</f>
+        <v/>
+      </c>
+      <c r="L32" s="158">
+        <f>SUM(F32:K32)</f>
+        <v/>
+      </c>
+      <c r="M32" s="158">
+        <f>SUM(M6:M30)</f>
+        <v/>
+      </c>
+      <c r="O32" s="155" t="inlineStr">
         <is>
           <t>UAH</t>
         </is>
       </c>
-      <c r="P30" s="155" t="inlineStr">
+      <c r="P32" s="155" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="F31">
-        <f>F30*41.2</f>
-        <v/>
-      </c>
-      <c r="G31">
-        <f>G30*41.2</f>
-        <v/>
-      </c>
-      <c r="H31">
-        <f>H30*41.2</f>
-        <v/>
-      </c>
-      <c r="I31">
-        <f>I30*41.2</f>
-        <v/>
-      </c>
-      <c r="J31">
-        <f>J30*41.2</f>
-        <v/>
-      </c>
-      <c r="K31">
-        <f>K30*41.2</f>
-        <v/>
-      </c>
-      <c r="L31">
-        <f>L30*41.2</f>
-        <v/>
-      </c>
-      <c r="M31">
-        <f>M30*41.2</f>
-        <v/>
-      </c>
-      <c r="N31" s="155" t="inlineStr">
+    <row r="33">
+      <c r="F33">
+        <f>F32*44.88</f>
+        <v/>
+      </c>
+      <c r="G33">
+        <f>G32*44.88</f>
+        <v/>
+      </c>
+      <c r="H33">
+        <f>H32*44.88</f>
+        <v/>
+      </c>
+      <c r="I33">
+        <f>I32*44.88</f>
+        <v/>
+      </c>
+      <c r="J33">
+        <f>J32*44.88</f>
+        <v/>
+      </c>
+      <c r="K33">
+        <f>K32*44.88</f>
+        <v/>
+      </c>
+      <c r="L33">
+        <f>L32*44.88</f>
+        <v/>
+      </c>
+      <c r="M33">
+        <f>M32*44.88</f>
+        <v/>
+      </c>
+      <c r="N33" s="155" t="inlineStr">
         <is>
           <t>CLIENT IN</t>
         </is>
       </c>
-      <c r="O31">
-        <f>P31*41.2</f>
-        <v/>
-      </c>
-      <c r="P31">
-        <f>M30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="N32" s="155" t="inlineStr">
-        <is>
-          <t>STUDIO (TAX)</t>
-        </is>
-      </c>
-      <c r="O32">
-        <f>P32*41.2</f>
-        <v/>
-      </c>
-      <c r="P32">
-        <f>P31-P31*0.05</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="N33" s="155" t="inlineStr">
-        <is>
-          <t>EMPL</t>
-        </is>
-      </c>
       <c r="O33">
-        <f>P33*41.2</f>
+        <f>P33*44.88</f>
         <v/>
       </c>
       <c r="P33">
-        <f>L30</f>
-        <v/>
+        <f>M32</f>
+        <v/>
+      </c>
+      <c r="Q33" s="155" t="inlineStr">
+        <is>
+          <t>TAX</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="N34" s="155" t="inlineStr">
         <is>
+          <t>STUDIO (TAX)</t>
+        </is>
+      </c>
+      <c r="O34">
+        <f>P34*44.88</f>
+        <v/>
+      </c>
+      <c r="P34">
+        <f>P33-P33*Q34</f>
+        <v/>
+      </c>
+      <c r="Q34" s="174" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="N35" s="155" t="inlineStr">
+        <is>
+          <t>EMPL</t>
+        </is>
+      </c>
+      <c r="O35">
+        <f>P35*44.88</f>
+        <v/>
+      </c>
+      <c r="P35">
+        <f>L32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="N36" s="155" t="inlineStr">
+        <is>
           <t>STUDIO</t>
         </is>
       </c>
-      <c r="O34">
-        <f>P34*41.2</f>
-        <v/>
-      </c>
-      <c r="P34">
-        <f>P32-P33</f>
+      <c r="O36">
+        <f>P36*44.88</f>
+        <v/>
+      </c>
+      <c r="P36">
+        <f>P34-P35</f>
         <v/>
       </c>
     </row>
@@ -3242,7 +3440,7 @@
       </c>
       <c r="B7" s="53" t="inlineStr">
         <is>
-          <t>Анастасі Верлинська - менеджер</t>
+          <t>Анастасія Верлинська - Line Producer</t>
         </is>
       </c>
       <c r="C7" s="112" t="n"/>
@@ -3269,7 +3467,7 @@
       </c>
       <c r="B8" s="53" t="inlineStr">
         <is>
-          <t>Анастасія Сиченко - тімлід</t>
+          <t>Анастасія Сиченко - Team Lead</t>
         </is>
       </c>
       <c r="C8" s="112" t="inlineStr">
@@ -3303,7 +3501,7 @@
       </c>
       <c r="B9" s="53" t="inlineStr">
         <is>
-          <t>Лащенко Сергій Олексійович</t>
+          <t>Лащенко Сергій Олексійович - Motion design</t>
         </is>
       </c>
       <c r="C9" s="112" t="inlineStr">
@@ -3344,7 +3542,7 @@
       </c>
       <c r="B10" s="53" t="inlineStr">
         <is>
-          <t>Терлецька Марія Максимівна</t>
+          <t>Терлецька Марія Максимівна - Motion design</t>
         </is>
       </c>
       <c r="E10" s="43" t="inlineStr">
@@ -3371,7 +3569,7 @@
       </c>
       <c r="B11" s="53" t="inlineStr">
         <is>
-          <t>Аліна Колесник</t>
+          <t>Аліна Колесник - Motion design</t>
         </is>
       </c>
       <c r="C11" s="54" t="n"/>
@@ -3390,7 +3588,7 @@
       </c>
       <c r="B12" s="150" t="inlineStr">
         <is>
-          <t>Злотко Олексій</t>
+          <t>Злотко Олексій - Motion design</t>
         </is>
       </c>
       <c r="C12" s="151" t="n"/>

</xml_diff>

<commit_message>
Rename MGX Excel seats from EMPL to LP / TL / MD.
Check sheets show TL 1, MD 1…; the calculator starts with LP 1. Leftover EMPL N headers on older tabs are rewritten the same way. board-update applies this on the live VPS files after restore.

Co-authored-by: lisenbart <lisenbart@gmail.com>
</commit_message>
<xml_diff>
--- a/data/finance/SUPERPLAY_MGX_Calculator.xlsx
+++ b/data/finance/SUPERPLAY_MGX_Calculator.xlsx
@@ -625,7 +625,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="40">
+  <fills count="41">
     <fill>
       <patternFill/>
     </fill>
@@ -848,6 +848,11 @@
         <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD9A8"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -877,7 +882,7 @@
     <xf numFmtId="0" fontId="58" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="58" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="223">
+  <cellXfs count="226">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1455,6 +1460,15 @@
     </xf>
     <xf numFmtId="49" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="1" xfId="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="85" fillId="40" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="84" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="84" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1755,32 +1769,32 @@
       </c>
       <c r="F5" s="204" t="inlineStr">
         <is>
-          <t>EMPL 1</t>
+          <t>LP 1</t>
         </is>
       </c>
       <c r="G5" s="204" t="inlineStr">
         <is>
-          <t>EMPL 2</t>
+          <t>TL 1</t>
         </is>
       </c>
       <c r="H5" s="204" t="inlineStr">
         <is>
-          <t>EMPL 3</t>
+          <t>MD 1</t>
         </is>
       </c>
       <c r="I5" s="204" t="inlineStr">
         <is>
-          <t>EMPL 4</t>
+          <t>MD 2</t>
         </is>
       </c>
       <c r="J5" s="204" t="inlineStr">
         <is>
-          <t>EMPL 5</t>
+          <t>MD 3</t>
         </is>
       </c>
       <c r="K5" s="204" t="inlineStr">
         <is>
-          <t>EMPL 6</t>
+          <t>MD 4</t>
         </is>
       </c>
       <c r="L5" s="204" t="inlineStr">
@@ -1809,7 +1823,7 @@
         <v/>
       </c>
       <c r="E6" s="205" t="n"/>
-      <c r="F6" s="207">
+      <c r="F6" s="223">
         <f>D6*5</f>
         <v/>
       </c>
@@ -1845,7 +1859,7 @@
         <v/>
       </c>
       <c r="E7" s="205" t="n"/>
-      <c r="F7" s="207">
+      <c r="F7" s="223">
         <f>D7*5</f>
         <v/>
       </c>
@@ -1881,7 +1895,7 @@
         <v/>
       </c>
       <c r="E8" s="205" t="n"/>
-      <c r="F8" s="207">
+      <c r="F8" s="223">
         <f>D8*5</f>
         <v/>
       </c>
@@ -1917,7 +1931,7 @@
         <v/>
       </c>
       <c r="E9" s="205" t="n"/>
-      <c r="F9" s="207">
+      <c r="F9" s="223">
         <f>D9*5</f>
         <v/>
       </c>
@@ -1953,7 +1967,7 @@
         <v/>
       </c>
       <c r="E10" s="205" t="n"/>
-      <c r="F10" s="207">
+      <c r="F10" s="223">
         <f>D10*5</f>
         <v/>
       </c>
@@ -1989,7 +2003,7 @@
         <v/>
       </c>
       <c r="E11" s="205" t="n"/>
-      <c r="F11" s="207">
+      <c r="F11" s="223">
         <f>D11*5</f>
         <v/>
       </c>
@@ -2025,7 +2039,7 @@
         <v/>
       </c>
       <c r="E12" s="205" t="n"/>
-      <c r="F12" s="207">
+      <c r="F12" s="223">
         <f>D12*5</f>
         <v/>
       </c>
@@ -2064,7 +2078,7 @@
         <v/>
       </c>
       <c r="E13" s="205" t="n"/>
-      <c r="F13" s="207">
+      <c r="F13" s="223">
         <f>D13*5</f>
         <v/>
       </c>
@@ -2100,7 +2114,7 @@
         <v/>
       </c>
       <c r="E14" s="205" t="n"/>
-      <c r="F14" s="207">
+      <c r="F14" s="223">
         <f>D14*5</f>
         <v/>
       </c>
@@ -2136,7 +2150,7 @@
         <v/>
       </c>
       <c r="E15" s="205" t="n"/>
-      <c r="F15" s="207">
+      <c r="F15" s="223">
         <f>D15*5</f>
         <v/>
       </c>
@@ -2172,7 +2186,7 @@
         <v/>
       </c>
       <c r="E16" s="205" t="n"/>
-      <c r="F16" s="207">
+      <c r="F16" s="223">
         <f>D16*5</f>
         <v/>
       </c>
@@ -2221,32 +2235,32 @@
       </c>
       <c r="F18" s="204" t="inlineStr">
         <is>
-          <t>EMPL 1</t>
+          <t>LP 1</t>
         </is>
       </c>
       <c r="G18" s="204" t="inlineStr">
         <is>
-          <t>EMPL 2</t>
+          <t>TL 1</t>
         </is>
       </c>
       <c r="H18" s="204" t="inlineStr">
         <is>
-          <t>EMPL 3</t>
+          <t>MD 1</t>
         </is>
       </c>
       <c r="I18" s="204" t="inlineStr">
         <is>
-          <t>EMPL 4</t>
+          <t>MD 2</t>
         </is>
       </c>
       <c r="J18" s="204" t="inlineStr">
         <is>
-          <t>EMPL 5</t>
+          <t>MD 3</t>
         </is>
       </c>
       <c r="K18" s="204" t="inlineStr">
         <is>
-          <t>EMPL 6</t>
+          <t>MD 4</t>
         </is>
       </c>
       <c r="L18" s="204" t="inlineStr">
@@ -2275,7 +2289,7 @@
         <v/>
       </c>
       <c r="E19" s="205" t="n"/>
-      <c r="F19" s="207">
+      <c r="F19" s="223">
         <f>D19*5</f>
         <v/>
       </c>
@@ -2311,7 +2325,7 @@
         <v/>
       </c>
       <c r="E20" s="205" t="n"/>
-      <c r="F20" s="207">
+      <c r="F20" s="223">
         <f>D20*5</f>
         <v/>
       </c>
@@ -2347,7 +2361,7 @@
         <v/>
       </c>
       <c r="E21" s="205" t="n"/>
-      <c r="F21" s="207">
+      <c r="F21" s="223">
         <f>D21*5</f>
         <v/>
       </c>
@@ -2383,7 +2397,7 @@
         <v/>
       </c>
       <c r="E22" s="205" t="n"/>
-      <c r="F22" s="207">
+      <c r="F22" s="223">
         <f>D22*5</f>
         <v/>
       </c>
@@ -2419,7 +2433,7 @@
         <v/>
       </c>
       <c r="E23" s="205" t="n"/>
-      <c r="F23" s="207">
+      <c r="F23" s="223">
         <f>D23*5</f>
         <v/>
       </c>
@@ -2455,7 +2469,7 @@
         <v/>
       </c>
       <c r="E24" s="205" t="n"/>
-      <c r="F24" s="207">
+      <c r="F24" s="223">
         <f>D24*5</f>
         <v/>
       </c>
@@ -2491,7 +2505,7 @@
         <v/>
       </c>
       <c r="E25" s="205" t="n"/>
-      <c r="F25" s="207">
+      <c r="F25" s="223">
         <f>D25*5</f>
         <v/>
       </c>
@@ -2527,7 +2541,7 @@
         <v/>
       </c>
       <c r="E26" s="205" t="n"/>
-      <c r="F26" s="207">
+      <c r="F26" s="223">
         <f>D26*5</f>
         <v/>
       </c>
@@ -2563,7 +2577,7 @@
         <v/>
       </c>
       <c r="E27" s="205" t="n"/>
-      <c r="F27" s="207">
+      <c r="F27" s="223">
         <f>D27*5</f>
         <v/>
       </c>
@@ -2599,7 +2613,7 @@
         <v/>
       </c>
       <c r="E28" s="205" t="n"/>
-      <c r="F28" s="207">
+      <c r="F28" s="223">
         <f>D28*5</f>
         <v/>
       </c>
@@ -2635,7 +2649,7 @@
         <v/>
       </c>
       <c r="E29" s="205" t="n"/>
-      <c r="F29" s="207">
+      <c r="F29" s="223">
         <f>D29*5</f>
         <v/>
       </c>
@@ -2671,7 +2685,7 @@
         <v/>
       </c>
       <c r="E30" s="205" t="n"/>
-      <c r="F30" s="207">
+      <c r="F30" s="223">
         <f>D30*5</f>
         <v/>
       </c>
@@ -2704,7 +2718,7 @@
         <v/>
       </c>
       <c r="E31" s="205" t="n"/>
-      <c r="F31" s="207">
+      <c r="F31" s="223">
         <f>D31*5</f>
         <v/>
       </c>
@@ -2737,7 +2751,7 @@
         <v/>
       </c>
       <c r="E32" s="205" t="n"/>
-      <c r="F32" s="207">
+      <c r="F32" s="223">
         <f>D32*5</f>
         <v/>
       </c>
@@ -2770,7 +2784,7 @@
         <v/>
       </c>
       <c r="E33" s="205" t="n"/>
-      <c r="F33" s="207">
+      <c r="F33" s="223">
         <f>D33*5</f>
         <v/>
       </c>
@@ -2849,35 +2863,35 @@
     </row>
     <row r="36">
       <c r="F36">
-        <f>F35*41.2</f>
+        <f>F35*44.7</f>
         <v/>
       </c>
       <c r="G36">
-        <f>G35*41.2</f>
+        <f>G35*44.7</f>
         <v/>
       </c>
       <c r="H36">
-        <f>H35*41.2</f>
+        <f>H35*44.7</f>
         <v/>
       </c>
       <c r="I36">
-        <f>I35*41.2</f>
+        <f>I35*44.7</f>
         <v/>
       </c>
       <c r="J36">
-        <f>J35*41.2</f>
+        <f>J35*44.7</f>
         <v/>
       </c>
       <c r="K36">
-        <f>K35*41.2</f>
+        <f>K35*44.7</f>
         <v/>
       </c>
       <c r="L36">
-        <f>L35*41.2</f>
+        <f>L35*44.7</f>
         <v/>
       </c>
       <c r="M36">
-        <f>M35*41.2</f>
+        <f>M35*44.7</f>
         <v/>
       </c>
       <c r="N36" s="201" t="inlineStr">
@@ -2886,7 +2900,7 @@
         </is>
       </c>
       <c r="O36">
-        <f>P36*41.2</f>
+        <f>P36*44.7</f>
         <v/>
       </c>
       <c r="P36">
@@ -2906,7 +2920,7 @@
         </is>
       </c>
       <c r="O37">
-        <f>P37*41.2</f>
+        <f>P37*44.7</f>
         <v/>
       </c>
       <c r="P37">
@@ -2924,7 +2938,7 @@
         </is>
       </c>
       <c r="O38">
-        <f>P38*41.2</f>
+        <f>P38*44.7</f>
         <v/>
       </c>
       <c r="P38">
@@ -2939,7 +2953,7 @@
         </is>
       </c>
       <c r="O39">
-        <f>P39*41.2</f>
+        <f>P39*44.7</f>
         <v/>
       </c>
       <c r="P39">
@@ -3047,34 +3061,34 @@
           <t>ADMIN</t>
         </is>
       </c>
-      <c r="F3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G3" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="H3" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="I3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="J3" s="31" t="inlineStr">
-        <is>
-          <t>Total EMPL</t>
-        </is>
-      </c>
-      <c r="K3" s="39" t="inlineStr">
-        <is>
-          <t>STUDIO</t>
+      <c r="F3" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G3" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H3" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I3" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J3" s="204" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K3" s="224" t="inlineStr">
+        <is>
+          <t>MD 4</t>
         </is>
       </c>
     </row>
@@ -4342,34 +4356,34 @@
           <t>ADMIN</t>
         </is>
       </c>
-      <c r="F3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G3" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="H3" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="I3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="J3" s="31" t="inlineStr">
-        <is>
-          <t>Total EMPL</t>
-        </is>
-      </c>
-      <c r="K3" s="39" t="inlineStr">
-        <is>
-          <t>STUDIO</t>
+      <c r="F3" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G3" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H3" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I3" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J3" s="204" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K3" s="224" t="inlineStr">
+        <is>
+          <t>MD 4</t>
         </is>
       </c>
     </row>
@@ -6014,34 +6028,34 @@
           <t>ADMIN</t>
         </is>
       </c>
-      <c r="F3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G3" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="H3" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="I3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="J3" s="31" t="inlineStr">
-        <is>
-          <t>Total EMPL</t>
-        </is>
-      </c>
-      <c r="K3" s="39" t="inlineStr">
-        <is>
-          <t>STUDIO</t>
+      <c r="F3" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G3" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H3" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I3" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J3" s="204" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K3" s="224" t="inlineStr">
+        <is>
+          <t>MD 4</t>
         </is>
       </c>
     </row>
@@ -7583,34 +7597,34 @@
           <t>ADMIN</t>
         </is>
       </c>
-      <c r="F5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="H5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="I5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="J5" s="31" t="inlineStr">
-        <is>
-          <t>Total EMPL</t>
-        </is>
-      </c>
-      <c r="K5" s="39" t="inlineStr">
-        <is>
-          <t>STUDIO</t>
+      <c r="F5" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G5" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H5" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I5" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J5" s="204" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K5" s="224" t="inlineStr">
+        <is>
+          <t>MD 4</t>
         </is>
       </c>
     </row>
@@ -8541,34 +8555,34 @@
           <t>ADMIN</t>
         </is>
       </c>
-      <c r="F5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="H5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="I5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="J5" s="31" t="inlineStr">
-        <is>
-          <t>Total EMPL</t>
-        </is>
-      </c>
-      <c r="K5" s="39" t="inlineStr">
-        <is>
-          <t>STUDIO</t>
+      <c r="F5" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G5" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H5" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I5" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J5" s="204" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K5" s="224" t="inlineStr">
+        <is>
+          <t>MD 4</t>
         </is>
       </c>
     </row>
@@ -9337,34 +9351,34 @@
           <t>ADMIN</t>
         </is>
       </c>
-      <c r="F5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="H5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="I5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="J5" s="31" t="inlineStr">
-        <is>
-          <t>Total EMPL</t>
-        </is>
-      </c>
-      <c r="K5" s="39" t="inlineStr">
-        <is>
-          <t>STUDIO</t>
+      <c r="F5" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G5" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H5" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I5" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J5" s="204" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K5" s="224" t="inlineStr">
+        <is>
+          <t>MD 4</t>
         </is>
       </c>
     </row>
@@ -10213,34 +10227,34 @@
           <t>ADMIN</t>
         </is>
       </c>
-      <c r="F5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="H5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="I5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="J5" s="31" t="inlineStr">
-        <is>
-          <t>Total EMPL</t>
-        </is>
-      </c>
-      <c r="K5" s="39" t="inlineStr">
-        <is>
-          <t>STUDIO</t>
+      <c r="F5" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G5" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H5" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I5" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J5" s="204" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K5" s="224" t="inlineStr">
+        <is>
+          <t>MD 4</t>
         </is>
       </c>
     </row>
@@ -11426,34 +11440,34 @@
         </is>
       </c>
       <c r="E5" s="25" t="n"/>
-      <c r="F5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="H5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="I5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="J5" s="31" t="inlineStr">
-        <is>
-          <t>Total EMPL</t>
-        </is>
-      </c>
-      <c r="K5" s="39" t="inlineStr">
-        <is>
-          <t>STUDIO</t>
+      <c r="F5" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G5" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H5" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I5" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J5" s="204" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K5" s="224" t="inlineStr">
+        <is>
+          <t>MD 4</t>
         </is>
       </c>
     </row>
@@ -12308,34 +12322,35 @@
           <t>HOURS</t>
         </is>
       </c>
-      <c r="E5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="F5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="G5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="H5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="I5" s="31" t="inlineStr">
-        <is>
-          <t>Total EMPL</t>
-        </is>
-      </c>
-      <c r="J5" s="39" t="inlineStr">
-        <is>
-          <t>STUDIO</t>
+      <c r="E5" s="204" t="n"/>
+      <c r="F5" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G5" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H5" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I5" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J5" s="224" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K5" s="204" t="inlineStr">
+        <is>
+          <t>MD 4</t>
         </is>
       </c>
     </row>
@@ -14244,34 +14259,35 @@
           <t>HOURS</t>
         </is>
       </c>
-      <c r="E5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="F5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="G5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="H5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="I5" s="31" t="inlineStr">
-        <is>
-          <t>Total EMPL</t>
-        </is>
-      </c>
-      <c r="J5" s="39" t="inlineStr">
-        <is>
-          <t>STUDIO</t>
+      <c r="E5" s="204" t="n"/>
+      <c r="F5" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G5" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H5" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I5" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J5" s="224" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K5" s="204" t="inlineStr">
+        <is>
+          <t>MD 4</t>
         </is>
       </c>
     </row>
@@ -19226,34 +19242,35 @@
           <t>HOURS</t>
         </is>
       </c>
-      <c r="E5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="F5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="G5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="H5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="I5" s="31" t="inlineStr">
-        <is>
-          <t>Total EMPL</t>
-        </is>
-      </c>
-      <c r="J5" s="39" t="inlineStr">
-        <is>
-          <t>STUDIO</t>
+      <c r="E5" s="204" t="n"/>
+      <c r="F5" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G5" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H5" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I5" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J5" s="224" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K5" s="204" t="inlineStr">
+        <is>
+          <t>MD 4</t>
         </is>
       </c>
     </row>
@@ -22368,34 +22385,35 @@
           <t>HOURS</t>
         </is>
       </c>
-      <c r="E5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="F5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="G5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="H5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="I5" s="31" t="inlineStr">
-        <is>
-          <t>Total EMPL</t>
-        </is>
-      </c>
-      <c r="J5" s="39" t="inlineStr">
-        <is>
-          <t>STUDIO</t>
+      <c r="E5" s="204" t="n"/>
+      <c r="F5" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G5" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H5" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I5" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J5" s="224" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K5" s="204" t="inlineStr">
+        <is>
+          <t>MD 4</t>
         </is>
       </c>
     </row>
@@ -24369,34 +24387,34 @@
           <t>D.LINE</t>
         </is>
       </c>
-      <c r="F5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="H5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="I5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="J5" s="31" t="inlineStr">
-        <is>
-          <t>Total EMPL</t>
-        </is>
-      </c>
-      <c r="K5" s="39" t="inlineStr">
-        <is>
-          <t>STUDIO</t>
+      <c r="F5" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G5" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H5" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I5" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J5" s="204" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K5" s="224" t="inlineStr">
+        <is>
+          <t>MD 4</t>
         </is>
       </c>
     </row>
@@ -25916,34 +25934,34 @@
           <t>D.LINE</t>
         </is>
       </c>
-      <c r="F5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="H5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="I5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="J5" s="31" t="inlineStr">
-        <is>
-          <t>Total EMPL</t>
-        </is>
-      </c>
-      <c r="K5" s="39" t="inlineStr">
-        <is>
-          <t>STUDIO</t>
+      <c r="F5" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G5" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H5" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I5" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J5" s="204" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K5" s="224" t="inlineStr">
+        <is>
+          <t>MD 4</t>
         </is>
       </c>
     </row>
@@ -27478,24 +27496,24 @@
           <t>D.LINE</t>
         </is>
       </c>
-      <c r="F5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="H5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="I5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
+      <c r="F5" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G5" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H5" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I5" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
         </is>
       </c>
       <c r="J5" s="31" t="inlineStr">
@@ -28834,6 +28852,7 @@
       <c r="H3" s="38" t="n"/>
       <c r="I3" s="38" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="111" t="inlineStr">
         <is>
@@ -28860,24 +28879,24 @@
           <t>D.LINE</t>
         </is>
       </c>
-      <c r="F5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="H5" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="I5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
+      <c r="F5" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G5" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H5" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I5" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
         </is>
       </c>
       <c r="J5" s="31" t="inlineStr">
@@ -31457,6 +31476,7 @@
       <c r="G96" s="33" t="n"/>
       <c r="K96" s="33" t="n"/>
     </row>
+    <row r="97"/>
     <row r="98">
       <c r="A98" s="11" t="n"/>
       <c r="B98" s="57" t="n"/>
@@ -31593,6 +31613,7 @@
       <c r="F3" s="38" t="n"/>
       <c r="G3" s="38" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="27" t="n"/>
       <c r="B5" s="23" t="inlineStr">
@@ -31615,14 +31636,14 @@
           <t>D.LINE</t>
         </is>
       </c>
-      <c r="F5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G5" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
+      <c r="F5" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G5" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
         </is>
       </c>
       <c r="H5" s="31" t="inlineStr">
@@ -32778,6 +32799,7 @@
         <v/>
       </c>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="A45" s="11" t="n"/>
       <c r="B45" s="57" t="n"/>
@@ -32837,7 +32859,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:Q38"/>
+  <dimension ref="A1:Q38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="3.6640625" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -32856,6 +32878,7 @@
     <col width="10.83203125" customWidth="1" style="1" min="15" max="16384"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="61" t="inlineStr">
         <is>
@@ -32907,14 +32930,14 @@
           <t>D.LINE</t>
         </is>
       </c>
-      <c r="F4" s="73" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="G4" s="73" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
+      <c r="F4" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G4" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
         </is>
       </c>
       <c r="H4" s="73" t="inlineStr">
@@ -33432,6 +33455,7 @@
       <c r="P18" s="4" t="n"/>
       <c r="Q18" s="4" t="n"/>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="P20" s="4" t="n"/>
       <c r="Q20" s="4" t="n"/>
@@ -33491,6 +33515,7 @@
       <c r="P28" s="4" t="n"/>
       <c r="Q28" s="4" t="n"/>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="M30" s="4" t="n"/>
       <c r="N30" s="4" t="n"/>
@@ -33504,6 +33529,10 @@
     <row r="32">
       <c r="K32" s="64" t="n"/>
     </row>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
     <row r="37">
       <c r="M37" s="4" t="n"/>
       <c r="N37" s="4" t="n"/>
@@ -33625,24 +33654,24 @@
           <t>D.LINE</t>
         </is>
       </c>
-      <c r="F4" s="72" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G4" s="73" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="H4" s="73" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="I4" s="74" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
+      <c r="F4" s="224" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G4" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H4" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I4" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
         </is>
       </c>
       <c r="J4" s="73" t="inlineStr">
@@ -33963,9 +33992,9 @@
         <f>SUM(K6:K11)</f>
         <v/>
       </c>
-      <c r="L12" s="80" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
+      <c r="L12" s="225" t="inlineStr">
+        <is>
+          <t>LP 1</t>
         </is>
       </c>
       <c r="M12" s="28">
@@ -33989,9 +34018,9 @@
       <c r="H13" s="12" t="n"/>
       <c r="I13" s="12" t="n"/>
       <c r="K13" s="10" t="n"/>
-      <c r="L13" s="32" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
+      <c r="L13" s="225" t="inlineStr">
+        <is>
+          <t>LP 1</t>
         </is>
       </c>
       <c r="M13" s="28">
@@ -34015,9 +34044,9 @@
       <c r="H14" s="12" t="n"/>
       <c r="I14" s="12" t="n"/>
       <c r="K14" s="10" t="n"/>
-      <c r="L14" s="32" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
+      <c r="L14" s="225" t="inlineStr">
+        <is>
+          <t>LP 1</t>
         </is>
       </c>
       <c r="M14" s="8">
@@ -34254,6 +34283,17 @@
         <v>17</v>
       </c>
     </row>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
     <row r="61">
       <c r="A61" s="11" t="n"/>
       <c r="B61" s="57" t="n"/>
@@ -37623,34 +37663,34 @@
           <t>ADMIN</t>
         </is>
       </c>
-      <c r="F2" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G2" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="H2" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="I2" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="J2" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 5</t>
-        </is>
-      </c>
-      <c r="K2" s="31" t="inlineStr">
-        <is>
-          <t>Total EMPL</t>
+      <c r="F2" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G2" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H2" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I2" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J2" s="204" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K2" s="204" t="inlineStr">
+        <is>
+          <t>MD 4</t>
         </is>
       </c>
       <c r="L2" s="39" t="inlineStr">
@@ -39427,34 +39467,34 @@
           <t>ADMIN</t>
         </is>
       </c>
-      <c r="F3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G3" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="H3" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="I3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="J3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 5</t>
-        </is>
-      </c>
-      <c r="K3" s="31" t="inlineStr">
-        <is>
-          <t>Total EMPL</t>
+      <c r="F3" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G3" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H3" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I3" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J3" s="204" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K3" s="204" t="inlineStr">
+        <is>
+          <t>MD 4</t>
         </is>
       </c>
       <c r="L3" s="39" t="inlineStr">
@@ -42219,34 +42259,34 @@
           <t>ADMIN</t>
         </is>
       </c>
-      <c r="F3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G3" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="H3" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="I3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="J3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 5</t>
-        </is>
-      </c>
-      <c r="K3" s="31" t="inlineStr">
-        <is>
-          <t>Total EMPL</t>
+      <c r="F3" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G3" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H3" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I3" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J3" s="204" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K3" s="204" t="inlineStr">
+        <is>
+          <t>MD 4</t>
         </is>
       </c>
       <c r="L3" s="39" t="inlineStr">
@@ -44458,34 +44498,34 @@
           <t>ADMIN</t>
         </is>
       </c>
-      <c r="F3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G3" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="H3" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="I3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="J3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 5</t>
-        </is>
-      </c>
-      <c r="K3" s="31" t="inlineStr">
-        <is>
-          <t>Total EMPL</t>
+      <c r="F3" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G3" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H3" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I3" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J3" s="204" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K3" s="204" t="inlineStr">
+        <is>
+          <t>MD 4</t>
         </is>
       </c>
       <c r="L3" s="39" t="inlineStr">
@@ -47235,34 +47275,34 @@
           <t>ADMIN</t>
         </is>
       </c>
-      <c r="F3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G3" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="H3" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="I3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="J3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 5</t>
-        </is>
-      </c>
-      <c r="K3" s="31" t="inlineStr">
-        <is>
-          <t>Total EMPL</t>
+      <c r="F3" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G3" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H3" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I3" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J3" s="204" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K3" s="204" t="inlineStr">
+        <is>
+          <t>MD 4</t>
         </is>
       </c>
       <c r="L3" s="39" t="inlineStr">
@@ -49073,41 +49113,37 @@
           <t>ADMIN</t>
         </is>
       </c>
-      <c r="F3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G3" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="H3" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="I3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="J3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 5</t>
-        </is>
-      </c>
-      <c r="K3" s="184" t="inlineStr">
-        <is>
-          <t>EMPL 6</t>
-        </is>
-      </c>
-      <c r="L3" s="184" t="inlineStr">
-        <is>
-          <t>EMPL 7</t>
-        </is>
-      </c>
+      <c r="F3" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G3" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H3" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I3" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J3" s="204" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K3" s="204" t="inlineStr">
+        <is>
+          <t>MD 4</t>
+        </is>
+      </c>
+      <c r="L3" s="204" t="n"/>
       <c r="M3" s="31" t="inlineStr">
         <is>
           <t>Total EMPL</t>
@@ -50035,41 +50071,37 @@
           <t>ADMIN</t>
         </is>
       </c>
-      <c r="F3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 1</t>
-        </is>
-      </c>
-      <c r="G3" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 2</t>
-        </is>
-      </c>
-      <c r="H3" s="110" t="inlineStr">
-        <is>
-          <t>EMPL 3</t>
-        </is>
-      </c>
-      <c r="I3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 4</t>
-        </is>
-      </c>
-      <c r="J3" s="98" t="inlineStr">
-        <is>
-          <t>EMPL 5</t>
-        </is>
-      </c>
-      <c r="K3" s="184" t="inlineStr">
-        <is>
-          <t>EMPL 6</t>
-        </is>
-      </c>
-      <c r="L3" s="184" t="inlineStr">
-        <is>
-          <t>EMPL 7</t>
-        </is>
-      </c>
+      <c r="F3" s="204" t="inlineStr">
+        <is>
+          <t>LP 1</t>
+        </is>
+      </c>
+      <c r="G3" s="204" t="inlineStr">
+        <is>
+          <t>TL 1</t>
+        </is>
+      </c>
+      <c r="H3" s="204" t="inlineStr">
+        <is>
+          <t>MD 1</t>
+        </is>
+      </c>
+      <c r="I3" s="204" t="inlineStr">
+        <is>
+          <t>MD 2</t>
+        </is>
+      </c>
+      <c r="J3" s="204" t="inlineStr">
+        <is>
+          <t>MD 3</t>
+        </is>
+      </c>
+      <c r="K3" s="204" t="inlineStr">
+        <is>
+          <t>MD 4</t>
+        </is>
+      </c>
+      <c r="L3" s="204" t="n"/>
       <c r="M3" s="31" t="inlineStr">
         <is>
           <t>Total EMPL</t>

</xml_diff>